<commit_message>
Cement policy levers round 3: output-based allocation, kiln performance standard, capacity replacement rule, clean-heat credit reach, carbon contract for difference, low-carbon procurement with blended cement, production tax credit, border fee, intensity standard, kiln fuel shift in source/target form, calcined clay plant capital, and a fifth pathway (electric kiln with CCS). The new pathway changes default results from 2037 (about 0.04 Mt CO2e lower in 2050); everything else is unchanged at defaults.
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
+++ b/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\ctrl-settings\GRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536016EB-9FB3-488A-8F82-734E939F6EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010EF132-B5FF-4879-9499-A50E3166BCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="698" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-17680" yWindow="1520" windowWidth="10480" windowHeight="8170" tabRatio="698" firstSheet="18" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,7 @@
     <sheet name="GRA-indstprocemiss" sheetId="20" r:id="rId16"/>
     <sheet name="GRA-hydgnprodsubs" sheetId="21" r:id="rId17"/>
     <sheet name="GRA-remainder" sheetId="16" r:id="rId18"/>
+    <sheet name="GRA-indstcleanmaterials" sheetId="24" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="69">
   <si>
     <t>GRA Government Revenue Accounting</t>
   </si>
@@ -257,6 +258,9 @@
   </si>
   <si>
     <t>harmless today since it evaluates to the intended 0, but do not copy that pattern). Deficit Spending = 5 matches all other industry subsidies.</t>
+  </si>
+  <si>
+    <t>industry clean materials support</t>
   </si>
 </sst>
 </file>
@@ -1493,6 +1497,71 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C5A4207-CDFC-4554-9385-3A1A13EAA63F}">
+  <sheetPr>
+    <tabColor theme="4" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2">
+        <f t="array" ref="B2:B6">TRANSPOSE('Set Values Here'!B15:F15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>

</xml_diff>